<commit_message>
updated the master sheet format
</commit_message>
<xml_diff>
--- a/assets/masterSheet_format.xlsx
+++ b/assets/masterSheet_format.xlsx
@@ -4,10 +4,11 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="21267" windowHeight="8019"/>
+    <workbookView windowWidth="21267" windowHeight="8019" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="19">
   <si>
     <t>SP No</t>
   </si>
@@ -52,19 +53,53 @@
   <si>
     <t>PLEASE DO NOT MAKE ANY CHANGES  TO THE COLUMN HEADERS OR SEQUENCE.
 COLUMNS MARKED RED ARE MANDATORY</t>
+  </si>
+  <si>
+    <t>Shift Name</t>
+  </si>
+  <si>
+    <t>In</t>
+  </si>
+  <si>
+    <t>Out</t>
+  </si>
+  <si>
+    <t>Deduct Lunch</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>W1</t>
+  </si>
+  <si>
+    <t>YES</t>
+  </si>
+  <si>
+    <t>G</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="180" formatCode="h:mm;@"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -81,6 +116,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
@@ -233,12 +275,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="37">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF434343"/>
+        <bgColor rgb="FF434343"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FFD9D9D9"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -248,12 +302,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF434343"/>
-        <bgColor rgb="FF434343"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.6"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -445,12 +493,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -571,55 +634,52 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -634,83 +694,92 @@
     <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1259,48 +1328,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
     </row>
     <row r="2" spans="9:13">
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="6"/>
+      <c r="L2" s="6"/>
+      <c r="M2" s="6"/>
     </row>
     <row r="3" spans="9:13">
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1309,4 +1378,104 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultColWidth="8.79279279279279" defaultRowHeight="14.4" outlineLevelRow="5" outlineLevelCol="3"/>
+  <cols>
+    <col min="4" max="4" width="21.4504504504505" customWidth="1"/>
+    <col min="5" max="5" width="19.3603603603604" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="C2" s="3">
+        <v>0.583333333333333</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="3">
+        <v>0.583333333333333</v>
+      </c>
+      <c r="C3" s="3">
+        <v>0.916666666666667</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="3">
+        <v>0.916666666666667</v>
+      </c>
+      <c r="C4" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="3">
+        <v>0.354166666666667</v>
+      </c>
+      <c r="C5" s="3">
+        <v>0.729166666666667</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="3">
+        <v>0.333333333333333</v>
+      </c>
+      <c r="C6" s="3">
+        <v>0.708333333333333</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
updated test data and mastersheet_upload.xlsx
</commit_message>
<xml_diff>
--- a/assets/masterSheet_format.xlsx
+++ b/assets/masterSheet_format.xlsx
@@ -4,11 +4,11 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="21267" windowHeight="8019" activeTab="1"/>
+    <workbookView windowWidth="21267" windowHeight="8019"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="employee_details" sheetId="1" r:id="rId1"/>
+    <sheet name="shift_definitions" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -51,8 +51,9 @@
     <t>Out OT Allowed</t>
   </si>
   <si>
-    <t>PLEASE DO NOT MAKE ANY CHANGES  TO THE COLUMN HEADERS OR SEQUENCE.
-COLUMNS MARKED RED ARE MANDATORY</t>
+    <t>1. PLEASE DO NOT MAKE ANY CHANGES  TO THE COLUMN HEADERS OR SEQUENCE.
+2. COLUMNS MARKED RED ARE MANDATORY.
+3. FORMAT ALL VALUES AS TEXT OR GENERAL.</t>
   </si>
   <si>
     <t>Shift Name</t>
@@ -780,7 +781,7 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1315,8 +1316,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:M3"/>
-  <sheetFormatPr defaultColWidth="8.79279279279279" defaultRowHeight="14.4" outlineLevelRow="2"/>
+  <dimension ref="A1:R4"/>
+  <sheetFormatPr defaultColWidth="8.79279279279279" defaultRowHeight="14.4" outlineLevelRow="3"/>
   <cols>
     <col min="1" max="1" width="5.89189189189189" customWidth="1"/>
     <col min="2" max="2" width="14.2792792792793" customWidth="1"/>
@@ -1327,7 +1328,7 @@
     <col min="7" max="7" width="13.5675675675676" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:18">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1356,24 +1357,51 @@
       <c r="K1" s="6"/>
       <c r="L1" s="6"/>
       <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6"/>
+      <c r="R1" s="6"/>
     </row>
-    <row r="2" spans="9:13">
+    <row r="2" spans="9:18">
       <c r="I2" s="6"/>
       <c r="J2" s="6"/>
       <c r="K2" s="6"/>
       <c r="L2" s="6"/>
       <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
+      <c r="O2" s="6"/>
+      <c r="P2" s="6"/>
+      <c r="Q2" s="6"/>
+      <c r="R2" s="6"/>
     </row>
-    <row r="3" spans="9:13">
+    <row r="3" spans="9:18">
       <c r="I3" s="6"/>
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>
       <c r="L3" s="6"/>
       <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
+      <c r="O3" s="6"/>
+      <c r="P3" s="6"/>
+      <c r="Q3" s="6"/>
+      <c r="R3" s="6"/>
+    </row>
+    <row r="4" spans="9:18">
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="I1:M3"/>
+    <mergeCell ref="I1:R4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>